<commit_message>
ADD: Main model results for both RF_prev and RF_prom.
</commit_message>
<xml_diff>
--- a/temporary_files/logit_highj_orthogonal_prom.xlsx
+++ b/temporary_files/logit_highj_orthogonal_prom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edgarduron/Documents/Working-Papers/AppStore-Research/AppStore_Analysis/AppStore/temporary_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54F9719-8C50-E04E-8361-6A4887345FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A40B535A-5462-C845-94BA-5AD0468C5E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="21520" windowHeight="14820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="21360" windowHeight="15560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -436,6 +436,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>